<commit_message>
entered first round of 2026 data!
</commit_message>
<xml_diff>
--- a/data/community_fall2026.xlsx
+++ b/data/community_fall2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernbromley/Desktop/AVCA_BANWR/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D069B2A0-359A-D542-A0F4-E0DF61D4E745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{056CC6C6-4146-184D-A3C0-310B7174B3CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28720" windowHeight="17160" xr2:uid="{7D6DEC84-1D80-5044-AEB0-AE046E367DDB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" xr2:uid="{7D6DEC84-1D80-5044-AEB0-AE046E367DDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,8 +38,53 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={CC52F66D-55DB-8E43-B0DE-51452FEF7967}</author>
+    <author>tc={CAF2C8A5-7E2B-F541-9DFB-700ACA44C592}</author>
+    <author>tc={AB0CE727-E125-8144-8002-E2E433E4C919}</author>
+    <author>tc={841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}</author>
+  </authors>
+  <commentList>
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{CC52F66D-55DB-8E43-B0DE-51452FEF7967}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    unk decussate forb!</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="1" shapeId="0" xr:uid="{CAF2C8A5-7E2B-F541-9DFB-700ACA44C592}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    unk aster w/ purple flowers!</t>
+      </text>
+    </comment>
+    <comment ref="AK1" authorId="2" shapeId="0" xr:uid="{AB0CE727-E125-8144-8002-E2E433E4C919}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    purpurea type</t>
+      </text>
+    </comment>
+    <comment ref="H7" authorId="3" shapeId="0" xr:uid="{841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    incl. Hairy panic</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>plot</t>
   </si>
@@ -72,19 +117,103 @@
   </si>
   <si>
     <t>ARITER</t>
+  </si>
+  <si>
+    <t>SALTRA</t>
+  </si>
+  <si>
+    <t>CHENOspp</t>
+  </si>
+  <si>
+    <t>CALERI</t>
+  </si>
+  <si>
+    <t>MACTAG</t>
+  </si>
+  <si>
+    <t>BOUGRA</t>
+  </si>
+  <si>
+    <t>PORTUspp</t>
+  </si>
+  <si>
+    <t>SIDAspp</t>
+  </si>
+  <si>
+    <t>DIGCAL</t>
+  </si>
+  <si>
+    <t>HEBOBS</t>
+  </si>
+  <si>
+    <t>SETARspp</t>
+  </si>
+  <si>
+    <t>IPOMOspp</t>
+  </si>
+  <si>
+    <t>KALLSspp</t>
+  </si>
+  <si>
+    <t>BOERHspp</t>
+  </si>
+  <si>
+    <t>ERIACU</t>
+  </si>
+  <si>
+    <t>HOPOBT</t>
+  </si>
+  <si>
+    <t>CROPUM</t>
+  </si>
+  <si>
+    <t>BOUERI</t>
+  </si>
+  <si>
+    <t>TALAUR</t>
+  </si>
+  <si>
+    <t>ARIWAT</t>
+  </si>
+  <si>
+    <t>GUTSAR</t>
+  </si>
+  <si>
+    <t>BIDENspp</t>
+  </si>
+  <si>
+    <t>SOLELA</t>
+  </si>
+  <si>
+    <t>DESCOV</t>
+  </si>
+  <si>
+    <t>ISOTEN</t>
+  </si>
+  <si>
+    <t>AMBCON</t>
+  </si>
+  <si>
+    <t>ARISTspp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -124,6 +253,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Bromley, Fern L - (fernb)" id="{C061624E-6404-7544-875D-2039BE9EB8DC}" userId="S::fernb@arizona.edu::30de849f-80a2-4b3d-a5a0-12893ddae609" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -441,12 +576,29 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="E1" dT="2026-08-31T16:45:58.29" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{CC52F66D-55DB-8E43-B0DE-51452FEF7967}">
+    <text>unk decussate forb!</text>
+  </threadedComment>
+  <threadedComment ref="O1" dT="2026-08-31T16:45:47.96" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{CAF2C8A5-7E2B-F541-9DFB-700ACA44C592}">
+    <text>unk aster w/ purple flowers!</text>
+  </threadedComment>
+  <threadedComment ref="AK1" dT="2026-08-31T18:09:06.76" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{AB0CE727-E125-8144-8002-E2E433E4C919}">
+    <text>purpurea type</text>
+  </threadedComment>
+  <threadedComment ref="H7" dT="2026-08-31T17:19:31.45" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}">
+    <text>incl. Hairy panic</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD559584-3F3E-3149-A2F9-E170630AB5BF}">
-  <dimension ref="A1:K3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD559584-3F3E-3149-A2F9-E170630AB5BF}">
+  <dimension ref="A1:AK26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -480,8 +632,86 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>97</v>
       </c>
@@ -515,11 +745,32 @@
       <c r="K2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>65</v>
       </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
       <c r="E3">
         <v>0.5</v>
       </c>
@@ -540,9 +791,575 @@
       </c>
       <c r="K3">
         <v>0.5</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>68</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>20</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0.5</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>74</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0.5</v>
+      </c>
+      <c r="N5">
+        <v>0.5</v>
+      </c>
+      <c r="O5">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>55</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>0.5</v>
+      </c>
+      <c r="I6">
+        <v>0.5</v>
+      </c>
+      <c r="M6">
+        <v>10</v>
+      </c>
+      <c r="P6">
+        <v>3</v>
+      </c>
+      <c r="Q6">
+        <v>0.5</v>
+      </c>
+      <c r="R6">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>61</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>0.5</v>
+      </c>
+      <c r="J7">
+        <v>0.5</v>
+      </c>
+      <c r="S7">
+        <v>10</v>
+      </c>
+      <c r="T7">
+        <v>0.5</v>
+      </c>
+      <c r="U7">
+        <v>0.5</v>
+      </c>
+      <c r="V7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>57</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
+      </c>
+      <c r="I8">
+        <v>0.5</v>
+      </c>
+      <c r="R8">
+        <v>0.5</v>
+      </c>
+      <c r="V8">
+        <v>10</v>
+      </c>
+      <c r="W8">
+        <v>3</v>
+      </c>
+      <c r="X8">
+        <v>0.5</v>
+      </c>
+      <c r="Y8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>84</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="M9">
+        <v>3</v>
+      </c>
+      <c r="Z9">
+        <v>3</v>
+      </c>
+      <c r="AA9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>94</v>
+      </c>
+      <c r="G10">
+        <v>0.5</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+      <c r="I10">
+        <v>10</v>
+      </c>
+      <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>3</v>
+      </c>
+      <c r="O10">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>67</v>
+      </c>
+      <c r="H11">
+        <v>0.5</v>
+      </c>
+      <c r="I11">
+        <v>10</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+      <c r="AB11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>88</v>
+      </c>
+      <c r="E12">
+        <v>0.5</v>
+      </c>
+      <c r="I12">
+        <v>3</v>
+      </c>
+      <c r="J12">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>91</v>
+      </c>
+      <c r="G13">
+        <v>0.5</v>
+      </c>
+      <c r="I13">
+        <v>20</v>
+      </c>
+      <c r="M13">
+        <v>0.5</v>
+      </c>
+      <c r="S13">
+        <v>0.5</v>
+      </c>
+      <c r="U13">
+        <v>0.5</v>
+      </c>
+      <c r="AC13">
+        <v>0.5</v>
+      </c>
+      <c r="AD13">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>63</v>
+      </c>
+      <c r="F14">
+        <v>10</v>
+      </c>
+      <c r="G14">
+        <v>0.5</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14">
+        <v>30</v>
+      </c>
+      <c r="R14">
+        <v>0.5</v>
+      </c>
+      <c r="U14">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>89</v>
+      </c>
+      <c r="F15">
+        <v>0.5</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>0.5</v>
+      </c>
+      <c r="M15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>49</v>
+      </c>
+      <c r="C16">
+        <v>0.5</v>
+      </c>
+      <c r="H16">
+        <v>0.5</v>
+      </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
+      <c r="O16">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>72</v>
+      </c>
+      <c r="I17">
+        <v>20</v>
+      </c>
+      <c r="J17">
+        <v>0.5</v>
+      </c>
+      <c r="R17">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>14</v>
+      </c>
+      <c r="H18">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>40</v>
+      </c>
+      <c r="I19">
+        <v>20</v>
+      </c>
+      <c r="J19">
+        <v>3</v>
+      </c>
+      <c r="O19">
+        <v>0.5</v>
+      </c>
+      <c r="S19">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>22</v>
+      </c>
+      <c r="F20">
+        <v>10</v>
+      </c>
+      <c r="G20">
+        <v>10</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="M20">
+        <v>10</v>
+      </c>
+      <c r="O20">
+        <v>30</v>
+      </c>
+      <c r="V20">
+        <v>3</v>
+      </c>
+      <c r="AB20">
+        <v>0.5</v>
+      </c>
+      <c r="AE20">
+        <v>0.5</v>
+      </c>
+      <c r="AF20">
+        <v>3</v>
+      </c>
+      <c r="AG20">
+        <v>0.5</v>
+      </c>
+      <c r="AH20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="H21">
+        <v>0.5</v>
+      </c>
+      <c r="I21">
+        <v>10</v>
+      </c>
+      <c r="J21">
+        <v>0.5</v>
+      </c>
+      <c r="K21">
+        <v>0.5</v>
+      </c>
+      <c r="L21">
+        <v>3</v>
+      </c>
+      <c r="R21">
+        <v>0.5</v>
+      </c>
+      <c r="AE21">
+        <v>3</v>
+      </c>
+      <c r="AI21">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>4</v>
+      </c>
+      <c r="B22">
+        <v>0.5</v>
+      </c>
+      <c r="H22">
+        <v>3</v>
+      </c>
+      <c r="I22">
+        <v>10</v>
+      </c>
+      <c r="J22">
+        <v>0.5</v>
+      </c>
+      <c r="AJ22">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>19</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>3</v>
+      </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
+      <c r="J23">
+        <v>0.5</v>
+      </c>
+      <c r="K23">
+        <v>0.5</v>
+      </c>
+      <c r="R23">
+        <v>0.5</v>
+      </c>
+      <c r="S23">
+        <v>3</v>
+      </c>
+      <c r="AE23">
+        <v>3</v>
+      </c>
+      <c r="AJ23">
+        <v>3</v>
+      </c>
+      <c r="AK23">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>26</v>
+      </c>
+      <c r="F24">
+        <v>3</v>
+      </c>
+      <c r="I24">
+        <v>30</v>
+      </c>
+      <c r="J24">
+        <v>0.5</v>
+      </c>
+      <c r="L24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>48</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="H25">
+        <v>0.5</v>
+      </c>
+      <c r="I25">
+        <v>10</v>
+      </c>
+      <c r="O25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>77</v>
+      </c>
+      <c r="H26">
+        <v>0.5</v>
+      </c>
+      <c r="I26">
+        <v>3</v>
+      </c>
+      <c r="J26">
+        <v>0.5</v>
+      </c>
+      <c r="L26">
+        <v>3</v>
+      </c>
+      <c r="O26">
+        <v>0.5</v>
+      </c>
+      <c r="AC26">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>